<commit_message>
Cereri de ofertă: antet completat cu expeditorul, contactul și data
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017cfyCLE359cmg5Q5QJewA2
</commit_message>
<xml_diff>
--- a/resurse/oferte/cereri/cerere-oferta-pepiniera-cobadin.xlsx
+++ b/resurse/oferte/cereri/cerere-oferta-pepiniera-cobadin.xlsx
@@ -491,14 +491,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>De la: ______________________ · telefon: ______________ · e-mail: ______________</t>
+          <t>De la: George Șerban · telefon: 0765468714 · e-mail: george357ro@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Data cererii: ____ . ____ . 2026</t>
+          <t>Data cererii: 6 octombrie 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Oferta Cobadin 2024–2025 salvată și transcrisă; cătina roșie rămâne la Cobadin, arțar tătăresc/scumpie/sâmbovină la Agigea, sânger la Selficom Galați
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017cfyCLE359cmg5Q5QJewA2
</commit_message>
<xml_diff>
--- a/resurse/oferte/cereri/cerere-oferta-pepiniera-cobadin.xlsx
+++ b/resurse/oferte/cereri/cerere-oferta-pepiniera-cobadin.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -571,16 +571,16 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Arțar tătăresc</t>
+          <t>Cătină roșie</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Acer tataricum</t>
+          <t>Tamarix ramosissima</t>
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
@@ -595,150 +595,34 @@
       <c r="H11" s="5" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Sâmbovină</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>Celtis australis</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="n">
-        <v>21</v>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>1–2 ani, 30–80 cm, rădăcină nudă sau ghiveci 1–2 l</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5">
-        <f>D12*F12</f>
+      <c r="A12" s="7" t="inlineStr"/>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr"/>
+      <c r="D12" s="7">
+        <f>SUM(D11:D11)</f>
         <v/>
       </c>
-      <c r="H12" s="5" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Sânger</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>Cornus sanguinea</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>38</v>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>1–2 ani, 30–80 cm, rădăcină nudă sau ghiveci 1–2 l</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5">
-        <f>D13*F13</f>
+      <c r="E12" s="7" t="inlineStr"/>
+      <c r="F12" s="7" t="inlineStr"/>
+      <c r="G12" s="7">
+        <f>SUM(G11:G11)</f>
         <v/>
       </c>
-      <c r="H13" s="5" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Scumpie</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>Cotinus coggygria</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="n">
-        <v>41</v>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>1–2 ani, 30–80 cm, rădăcină nudă sau ghiveci 1–2 l</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5">
-        <f>D14*F14</f>
-        <v/>
-      </c>
-      <c r="H14" s="5" t="n"/>
+      <c r="H12" s="7" t="inlineStr"/>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Vă rugăm să precizați: costul transportului la Crucea sau adresa de ridicare, termenul de valabilitate al ofertei, dacă puteți rezerva cantitățile până la confirmare, și eventualele specii pe care nu le aveți (cu propuneri de înlocuire).</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Cătină roșie</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>Tamarix ramosissima</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>1–2 ani, 30–80 cm, rădăcină nudă sau ghiveci 1–2 l</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5">
-        <f>D15*F15</f>
-        <v/>
-      </c>
-      <c r="H15" s="5" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr"/>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr"/>
-      <c r="D16" s="7">
-        <f>SUM(D11:D15)</f>
-        <v/>
-      </c>
-      <c r="E16" s="7" t="inlineStr"/>
-      <c r="F16" s="7" t="inlineStr"/>
-      <c r="G16" s="7">
-        <f>SUM(G11:G15)</f>
-        <v/>
-      </c>
-      <c r="H16" s="7" t="inlineStr"/>
-    </row>
-    <row r="18" ht="45" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Vă rugăm să precizați: costul transportului la Crucea sau adresa de ridicare, termenul de valabilitate al ofertei, dacă puteți rezerva cantitățile până la confirmare, și eventualele specii pe care nu le aveți (cu propuneri de înlocuire).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Vă mulțumim.</t>
         </is>
@@ -748,8 +632,8 @@
   <mergeCells count="4">
     <mergeCell ref="A7:H7"/>
     <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A14:H14"/>
     <mergeCell ref="A6:H6"/>
-    <mergeCell ref="A18:H18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>

</xml_diff>